<commit_message>
chore: organize repository and detail contribution records
</commit_message>
<xml_diff>
--- a/version2/Contribution(1).xlsx
+++ b/version2/Contribution(1).xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="example1" sheetId="2" r:id="R9e31aac06d2f47f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="example1" sheetId="2" r:id="Ra2aa9b929f66440a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1171,7 +1171,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E7" s="21" t="str">
-        <x:v>Workshop task ownership</x:v>
+        <x:v>Confirmed individual contribution</x:v>
       </x:c>
       <x:c r="F7" s="20" t="s">
         <x:v>8</x:v>
@@ -1180,7 +1180,7 @@
         <x:v>9</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" s="5" customFormat="1" ht="168" customHeight="1">
+    <x:row r="8" s="5" customFormat="1" ht="234" customHeight="1">
       <x:c r="A8" s="14" t="s">
         <x:v>10</x:v>
       </x:c>
@@ -1194,16 +1194,17 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>First owner
-T01 (PB01) Reconcile requirement identifiers
-T02 (PB01) Record rules and scope assumptions
-T04 (PB03) Verify referral decisions and correlation
-T07 (PB05) Verify consent and request forms
-T10 (PB07) Repair stop and change ordering
-T22 (PB16) Assess requirement support and gaps
-T26 (PB19) Record standups reviews and handovers
-Second owner: T03, T08, T09, T11, T18, T19, T20, T21.
-Individual completion evidence: pending confirmation.</x:v>
+        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
+PB01 Requirements and assumptions
+Scope: Case requirements, business rules, scope assumptions and traceability.
+PB02 Operational patient pathway
+Scope: Main patient pathway, process lanes and event subprocess structure.
+PB03 Referral review
+Scope: Referral receipt, document checks, suitability decisions and referral correlation.
+PB04 Appointments and patient contact
+Scope: Appointment booking, telephone contact, rescheduling and cancellation.
+PB05 Consent and treatment authorisation
+Scope: Clinical assessment, consent and authorised treatment-request information.</x:v>
       </x:c>
       <x:c r="F8" s="17" t="n">
         <x:v>0.26</x:v>
@@ -1222,7 +1223,7 @@
       <x:c r="F9" s="19"/>
       <x:c r="G9" s="9"/>
     </x:row>
-    <x:row r="10" s="5" customFormat="1" ht="196" customHeight="1">
+    <x:row r="10" s="5" customFormat="1" ht="234" customHeight="1">
       <x:c r="A10" s="14" t="s">
         <x:v>13</x:v>
       </x:c>
@@ -1236,18 +1237,17 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E10" s="26" t="str">
-        <x:v>First owner
-T14 (PB11) Review current acceptance plan
-T15 (PB12) Identify integrated baseline
-T16 (PB12) Integrate approved version2 fixes
-T19 (PB15) Review SD dependencies
-T20 (PB15) Review SR refinements and applicability
-T21 (PB15) Align models and record feedback
-T23 (PB17) Preserve baseline acceptance results
-T24 (PB17) Retest the integrated current version
-T27 (PB20) Verify SP05 HTTP contract and recovery
-Second owner: T07, T12, T13, T17, T25, T26.
-Individual completion evidence: pending confirmation.</x:v>
+        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
+PB09 Patient enquiries
+Scope: Administrative, clinical and financial enquiry routing and recorded outcomes.
+PB10 Access audit and recovery
+Scope: Role boundaries, access audit, downtime and restoration correlation.
+PB11 Acceptance test plan
+Scope: Requirement-to-test mapping, original acceptance criteria and test-version boundaries.
+PB12 Version integration
+Scope: Model, form and Worker alignment, deployment identity and version integration.
+PB13 Reports and communication preferences
+Scope: Reporting information, data sources and patient communication preferences.</x:v>
       </x:c>
       <x:c r="F10" s="17" t="n">
         <x:v>0.26</x:v>
@@ -1266,7 +1266,7 @@
       <x:c r="F11" s="19"/>
       <x:c r="G11" s="9"/>
     </x:row>
-    <x:row r="12" s="5" customFormat="1" ht="126" customHeight="1">
+    <x:row r="12" s="5" customFormat="1" ht="312" customHeight="1">
       <x:c r="A12" s="14" t="s">
         <x:v>16</x:v>
       </x:c>
@@ -1280,13 +1280,21 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>First owner
-T11 (PB08) Repair letter reminders and isolation
-T12 (PB09) Verify enquiry routing and closure
-T17 (PB13) Specify reports and communication needs
-T25 (PB18) Prepare demonstration and decisions
-Second owner: T04, T05, T06, T15, T16, T22.
-Individual completion evidence: pending confirmation.</x:v>
+        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
+PB14 Strategic BPMN
+Scope: Business-level process modelling and mapping to operational processes.
+PB15 Integrated iStar SD and SR
+Scope: Actor dependencies, goals, tasks, refinements and integrated model alignment.
+PB16 Requirements consistency assessment
+Scope: Consistency between requirements, BPMN and strategic models; support and gap mapping.
+PB17 Acceptance execution and evaluation
+Scope: Acceptance scenarios, frozen baselines, retesting and interpretation of results.
+PB18 Demonstration and decisions
+Scope: SP05 request flow, availability outcomes, failure handling and design decisions.
+PB19 Agile records and handovers
+Scope: Task coordination, review feedback, contribution records and handover information.
+PB20 SP05 external availability and recovery
+Scope: External availability request, boolean response mapping, pending capacity and HTTP failure recovery.</x:v>
       </x:c>
       <x:c r="F12" s="17" t="n">
         <x:v>0.23</x:v>
@@ -1305,7 +1313,7 @@
       <x:c r="F13" s="19"/>
       <x:c r="G13" s="9"/>
     </x:row>
-    <x:row r="14" s="5" customFormat="1" ht="168" customHeight="1">
+    <x:row r="14" s="5" customFormat="1" ht="156" customHeight="1">
       <x:c r="A14" s="14" t="s">
         <x:v>19</x:v>
       </x:c>
@@ -1319,16 +1327,13 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="E14" s="26" t="str">
-        <x:v>First owner
-T03 (PB02) Maintain current process and lanes
-T05 (PB04) Implement date and contact guards
-T06 (PB04) Verify changes and cancellation
-T08 (PB06) Complete funding and payment guards
-T09 (PB06) Enforce refund and transfer rules
-T13 (PB10) Verify permissions audit and restoration
-T18 (PB14) Review strategic BPMN deliverable
-Second owner: T01, T02, T10, T14, T23, T24, T27.
-Individual completion evidence: pending confirmation.</x:v>
+        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
+PB06 Funding payments and refunds
+Scope: Funding decisions, payment handling, refunds and transfer routes.
+PB07 Treatment review and changes
+Scope: Fitness review, clinical stops, treatment changes and financial rechecks.
+PB08 Clinic letters and reminders
+Scope: Letter drafting, consultant approval, administrative processing and reminders.</x:v>
       </x:c>
       <x:c r="F14" s="17" t="n">
         <x:v>0.25</x:v>
@@ -1354,7 +1359,7 @@
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
       <x:c r="A16" s="29" t="str">
-        <x:v>Source: Agile Workshop.docx, Version 2, Parts 3 and 4. Churchill = Songjie Qiu (23084419). cyc = Chenyu Yang (23084439).</x:v>
+        <x:v>Authorship confirmed by the team on 20 October 2026. Churchill = Songjie Qiu (23084419); cyc/CYC = Chenyu Yang (23084439).</x:v>
       </x:c>
       <x:c r="B16" s="29"/>
       <x:c r="C16" s="29"/>
@@ -1365,7 +1370,7 @@
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
       <x:c r="A17" s="29" t="str">
-        <x:v>Tasks show first-owner and second-owner assignments. Personal completion evidence remains to be confirmed. Contribution percentages are the specified allocation, not a calculation from workshop estimates.</x:v>
+        <x:v>PB descriptions identify functional scope, not acceptance-test completion. Workshop review/fix owners are separate from original authors. The agreed percentages remain unchanged.</x:v>
       </x:c>
       <x:c r="B17" s="29"/>
       <x:c r="C17" s="29"/>

</xml_diff>

<commit_message>
chore: organize repository and detail contribution records (#6)
Co-authored-by: heavenyyy <13380669020@qq.com>
</commit_message>
<xml_diff>
--- a/version2/Contribution(1).xlsx
+++ b/version2/Contribution(1).xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="example1" sheetId="2" r:id="R9e31aac06d2f47f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="example1" sheetId="2" r:id="Ra2aa9b929f66440a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1171,7 +1171,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E7" s="21" t="str">
-        <x:v>Workshop task ownership</x:v>
+        <x:v>Confirmed individual contribution</x:v>
       </x:c>
       <x:c r="F7" s="20" t="s">
         <x:v>8</x:v>
@@ -1180,7 +1180,7 @@
         <x:v>9</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" s="5" customFormat="1" ht="168" customHeight="1">
+    <x:row r="8" s="5" customFormat="1" ht="234" customHeight="1">
       <x:c r="A8" s="14" t="s">
         <x:v>10</x:v>
       </x:c>
@@ -1194,16 +1194,17 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>First owner
-T01 (PB01) Reconcile requirement identifiers
-T02 (PB01) Record rules and scope assumptions
-T04 (PB03) Verify referral decisions and correlation
-T07 (PB05) Verify consent and request forms
-T10 (PB07) Repair stop and change ordering
-T22 (PB16) Assess requirement support and gaps
-T26 (PB19) Record standups reviews and handovers
-Second owner: T03, T08, T09, T11, T18, T19, T20, T21.
-Individual completion evidence: pending confirmation.</x:v>
+        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
+PB01 Requirements and assumptions
+Scope: Case requirements, business rules, scope assumptions and traceability.
+PB02 Operational patient pathway
+Scope: Main patient pathway, process lanes and event subprocess structure.
+PB03 Referral review
+Scope: Referral receipt, document checks, suitability decisions and referral correlation.
+PB04 Appointments and patient contact
+Scope: Appointment booking, telephone contact, rescheduling and cancellation.
+PB05 Consent and treatment authorisation
+Scope: Clinical assessment, consent and authorised treatment-request information.</x:v>
       </x:c>
       <x:c r="F8" s="17" t="n">
         <x:v>0.26</x:v>
@@ -1222,7 +1223,7 @@
       <x:c r="F9" s="19"/>
       <x:c r="G9" s="9"/>
     </x:row>
-    <x:row r="10" s="5" customFormat="1" ht="196" customHeight="1">
+    <x:row r="10" s="5" customFormat="1" ht="234" customHeight="1">
       <x:c r="A10" s="14" t="s">
         <x:v>13</x:v>
       </x:c>
@@ -1236,18 +1237,17 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E10" s="26" t="str">
-        <x:v>First owner
-T14 (PB11) Review current acceptance plan
-T15 (PB12) Identify integrated baseline
-T16 (PB12) Integrate approved version2 fixes
-T19 (PB15) Review SD dependencies
-T20 (PB15) Review SR refinements and applicability
-T21 (PB15) Align models and record feedback
-T23 (PB17) Preserve baseline acceptance results
-T24 (PB17) Retest the integrated current version
-T27 (PB20) Verify SP05 HTTP contract and recovery
-Second owner: T07, T12, T13, T17, T25, T26.
-Individual completion evidence: pending confirmation.</x:v>
+        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
+PB09 Patient enquiries
+Scope: Administrative, clinical and financial enquiry routing and recorded outcomes.
+PB10 Access audit and recovery
+Scope: Role boundaries, access audit, downtime and restoration correlation.
+PB11 Acceptance test plan
+Scope: Requirement-to-test mapping, original acceptance criteria and test-version boundaries.
+PB12 Version integration
+Scope: Model, form and Worker alignment, deployment identity and version integration.
+PB13 Reports and communication preferences
+Scope: Reporting information, data sources and patient communication preferences.</x:v>
       </x:c>
       <x:c r="F10" s="17" t="n">
         <x:v>0.26</x:v>
@@ -1266,7 +1266,7 @@
       <x:c r="F11" s="19"/>
       <x:c r="G11" s="9"/>
     </x:row>
-    <x:row r="12" s="5" customFormat="1" ht="126" customHeight="1">
+    <x:row r="12" s="5" customFormat="1" ht="312" customHeight="1">
       <x:c r="A12" s="14" t="s">
         <x:v>16</x:v>
       </x:c>
@@ -1280,13 +1280,21 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>First owner
-T11 (PB08) Repair letter reminders and isolation
-T12 (PB09) Verify enquiry routing and closure
-T17 (PB13) Specify reports and communication needs
-T25 (PB18) Prepare demonstration and decisions
-Second owner: T04, T05, T06, T15, T16, T22.
-Individual completion evidence: pending confirmation.</x:v>
+        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
+PB14 Strategic BPMN
+Scope: Business-level process modelling and mapping to operational processes.
+PB15 Integrated iStar SD and SR
+Scope: Actor dependencies, goals, tasks, refinements and integrated model alignment.
+PB16 Requirements consistency assessment
+Scope: Consistency between requirements, BPMN and strategic models; support and gap mapping.
+PB17 Acceptance execution and evaluation
+Scope: Acceptance scenarios, frozen baselines, retesting and interpretation of results.
+PB18 Demonstration and decisions
+Scope: SP05 request flow, availability outcomes, failure handling and design decisions.
+PB19 Agile records and handovers
+Scope: Task coordination, review feedback, contribution records and handover information.
+PB20 SP05 external availability and recovery
+Scope: External availability request, boolean response mapping, pending capacity and HTTP failure recovery.</x:v>
       </x:c>
       <x:c r="F12" s="17" t="n">
         <x:v>0.23</x:v>
@@ -1305,7 +1313,7 @@
       <x:c r="F13" s="19"/>
       <x:c r="G13" s="9"/>
     </x:row>
-    <x:row r="14" s="5" customFormat="1" ht="168" customHeight="1">
+    <x:row r="14" s="5" customFormat="1" ht="156" customHeight="1">
       <x:c r="A14" s="14" t="s">
         <x:v>19</x:v>
       </x:c>
@@ -1319,16 +1327,13 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="E14" s="26" t="str">
-        <x:v>First owner
-T03 (PB02) Maintain current process and lanes
-T05 (PB04) Implement date and contact guards
-T06 (PB04) Verify changes and cancellation
-T08 (PB06) Complete funding and payment guards
-T09 (PB06) Enforce refund and transfer rules
-T13 (PB10) Verify permissions audit and restoration
-T18 (PB14) Review strategic BPMN deliverable
-Second owner: T01, T02, T10, T14, T23, T24, T27.
-Individual completion evidence: pending confirmation.</x:v>
+        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
+PB06 Funding payments and refunds
+Scope: Funding decisions, payment handling, refunds and transfer routes.
+PB07 Treatment review and changes
+Scope: Fitness review, clinical stops, treatment changes and financial rechecks.
+PB08 Clinic letters and reminders
+Scope: Letter drafting, consultant approval, administrative processing and reminders.</x:v>
       </x:c>
       <x:c r="F14" s="17" t="n">
         <x:v>0.25</x:v>
@@ -1354,7 +1359,7 @@
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
       <x:c r="A16" s="29" t="str">
-        <x:v>Source: Agile Workshop.docx, Version 2, Parts 3 and 4. Churchill = Songjie Qiu (23084419). cyc = Chenyu Yang (23084439).</x:v>
+        <x:v>Authorship confirmed by the team on 20 October 2026. Churchill = Songjie Qiu (23084419); cyc/CYC = Chenyu Yang (23084439).</x:v>
       </x:c>
       <x:c r="B16" s="29"/>
       <x:c r="C16" s="29"/>
@@ -1365,7 +1370,7 @@
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
       <x:c r="A17" s="29" t="str">
-        <x:v>Tasks show first-owner and second-owner assignments. Personal completion evidence remains to be confirmed. Contribution percentages are the specified allocation, not a calculation from workshop estimates.</x:v>
+        <x:v>PB descriptions identify functional scope, not acceptance-test completion. Workshop review/fix owners are separate from original authors. The agreed percentages remain unchanged.</x:v>
       </x:c>
       <x:c r="B17" s="29"/>
       <x:c r="C17" s="29"/>

</xml_diff>

<commit_message>
docs: map contributions to the 16 business activities
</commit_message>
<xml_diff>
--- a/version2/Contribution(1).xlsx
+++ b/version2/Contribution(1).xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="example1" sheetId="2" r:id="Ra2aa9b929f66440a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="example1" sheetId="2" r:id="Rdaeb859c48e841f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1180,7 +1180,7 @@
         <x:v>9</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" s="5" customFormat="1" ht="234" customHeight="1">
+    <x:row r="8" s="5" customFormat="1" ht="150" customHeight="1">
       <x:c r="A8" s="14" t="s">
         <x:v>10</x:v>
       </x:c>
@@ -1194,17 +1194,12 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
-PB01 Requirements and assumptions
-Scope: Case requirements, business rules, scope assumptions and traceability.
-PB02 Operational patient pathway
-Scope: Main patient pathway, process lanes and event subprocess structure.
-PB03 Referral review
-Scope: Referral receipt, document checks, suitability decisions and referral correlation.
-PB04 Appointments and patient contact
-Scope: Appointment booking, telephone contact, rescheduling and cancellation.
-PB05 Consent and treatment authorisation
-Scope: Clinical assessment, consent and authorised treatment-request information.</x:v>
+        <x:v>Authored the BPMN, SD/SR, Worker implementation and strategic-model portions for these business activities:
+1. Receive referrals, check supporting documents and request missing information.
+2. Review referrals clinically and accept, reject, redirect or request more information.
+3. Book new-patient appointments, contact patients and record contact outcomes.
+4. Conduct consultations, diagnose, discuss treatment, record consent and authorise treatment requests.
+5. Coordinate treatment and chemotherapy bookings, resources and external services.</x:v>
       </x:c>
       <x:c r="F8" s="17" t="n">
         <x:v>0.26</x:v>
@@ -1223,7 +1218,7 @@
       <x:c r="F9" s="19"/>
       <x:c r="G9" s="9"/>
     </x:row>
-    <x:row r="10" s="5" customFormat="1" ht="234" customHeight="1">
+    <x:row r="10" s="5" customFormat="1" ht="135" customHeight="1">
       <x:c r="A10" s="14" t="s">
         <x:v>13</x:v>
       </x:c>
@@ -1237,17 +1232,12 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E10" s="26" t="str">
-        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
-PB09 Patient enquiries
-Scope: Administrative, clinical and financial enquiry routing and recorded outcomes.
-PB10 Access audit and recovery
-Scope: Role boundaries, access audit, downtime and restoration correlation.
-PB11 Acceptance test plan
-Scope: Requirement-to-test mapping, original acceptance criteria and test-version boundaries.
-PB12 Version integration
-Scope: Model, form and Worker alignment, deployment identity and version integration.
-PB13 Reports and communication preferences
-Scope: Reporting information, data sources and patient communication preferences.</x:v>
+        <x:v>Authored the BPMN, SD/SR, Worker implementation and strategic-model portions for these business activities:
+9. Authorise and manage treatment changes, postponements and urgent exceptions.
+10. Manage cancellations, declined appointments and non-attendance, including clinical review.
+11. Review payment transfers and approve, process and record refunds.
+12. Record, classify, prioritise, route and resolve patient enquiries.
+13. Prepare, approve, check and distribute clinic letters; monitor delays and escalate them.</x:v>
       </x:c>
       <x:c r="F10" s="17" t="n">
         <x:v>0.26</x:v>
@@ -1266,7 +1256,7 @@
       <x:c r="F11" s="19"/>
       <x:c r="G11" s="9"/>
     </x:row>
-    <x:row r="12" s="5" customFormat="1" ht="312" customHeight="1">
+    <x:row r="12" s="5" customFormat="1" ht="120" customHeight="1">
       <x:c r="A12" s="14" t="s">
         <x:v>16</x:v>
       </x:c>
@@ -1280,21 +1270,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
-PB14 Strategic BPMN
-Scope: Business-level process modelling and mapping to operational processes.
-PB15 Integrated iStar SD and SR
-Scope: Actor dependencies, goals, tasks, refinements and integrated model alignment.
-PB16 Requirements consistency assessment
-Scope: Consistency between requirements, BPMN and strategic models; support and gap mapping.
-PB17 Acceptance execution and evaluation
-Scope: Acceptance scenarios, frozen baselines, retesting and interpretation of results.
-PB18 Demonstration and decisions
-Scope: SP05 request flow, availability outcomes, failure handling and design decisions.
-PB19 Agile records and handovers
-Scope: Task coordination, review feedback, contribution records and handover information.
-PB20 SP05 external availability and recovery
-Scope: External availability request, boolean response mapping, pending capacity and HTTP failure recovery.</x:v>
+        <x:v>Authored the BPMN, SD/SR, Worker implementation and strategic-model portions for these business activities:
+14. Request and book follow-up appointments and communicate arrangements.
+15. Monitor patient pathways and produce operational and financial reports.
+16. Maintain patient identity and records, control access, preserve audit trails and manage service outages.</x:v>
       </x:c>
       <x:c r="F12" s="17" t="n">
         <x:v>0.23</x:v>
@@ -1313,7 +1292,7 @@
       <x:c r="F13" s="19"/>
       <x:c r="G13" s="9"/>
     </x:row>
-    <x:row r="14" s="5" customFormat="1" ht="156" customHeight="1">
+    <x:row r="14" s="5" customFormat="1" ht="120" customHeight="1">
       <x:c r="A14" s="14" t="s">
         <x:v>19</x:v>
       </x:c>
@@ -1327,13 +1306,10 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="E14" s="26" t="str">
-        <x:v>Authored the related BPMN, SD/SR, Worker implementation and strategic-model sections:
-PB06 Funding payments and refunds
-Scope: Funding decisions, payment handling, refunds and transfer routes.
-PB07 Treatment review and changes
-Scope: Fitness review, clinical stops, treatment changes and financial rechecks.
-PB08 Clinic letters and reminders
-Scope: Letter drafting, consultant approval, administrative processing and reminders.</x:v>
+        <x:v>Authored the BPMN, SD/SR, Worker implementation and strategic-model portions for these business activities:
+6. Check funding eligibility, obtain funding approval and determine applicable charges.
+7. Request payments, record outcomes and investigate failed, duplicate or unconfirmed transactions.
+8. Deliver treatment, arrange tests and reviews, and assess fitness for further cycles.</x:v>
       </x:c>
       <x:c r="F14" s="17" t="n">
         <x:v>0.25</x:v>
@@ -1359,7 +1335,7 @@
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
       <x:c r="A16" s="29" t="str">
-        <x:v>Authorship confirmed by the team on 20 October 2026. Churchill = Songjie Qiu (23084419); cyc/CYC = Chenyu Yang (23084439).</x:v>
+        <x:v>Source: team-confirmed authorship and the 16 numbered business activities in the case study, clarified on 20 October 2026.</x:v>
       </x:c>
       <x:c r="B16" s="29"/>
       <x:c r="C16" s="29"/>
@@ -1370,7 +1346,7 @@
     </x:row>
     <x:row r="17" ht="32" customHeight="1">
       <x:c r="A17" s="29" t="str">
-        <x:v>PB descriptions identify functional scope, not acceptance-test completion. Workshop review/fix owners are separate from original authors. The agreed percentages remain unchanged.</x:v>
+        <x:v>Numbers 1-16 refer to business activities, not Workshop PB01-PB20. Authorship does not imply all acceptance criteria passed. Agreed contribution percentages remain unchanged.</x:v>
       </x:c>
       <x:c r="B17" s="29"/>
       <x:c r="C17" s="29"/>

</xml_diff>